<commit_message>
Update code, figures and results for  submission
</commit_message>
<xml_diff>
--- a/result/clustering_performance_scRNA.xlsx
+++ b/result/clustering_performance_scRNA.xlsx
@@ -1,22 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjyan\Desktop\ppt\ppt-2026年\文章素材\文章正文\scGEM_benchmark\result\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jjyan\Documents\GitHub\scGEM_benchmark_NCS\result\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5858EE6-495C-4354-9B77-2328ED400A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89684E1A-A1E0-4EE5-8E6B-BFA4DF7AF1DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-1155" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10680" yWindow="2475" windowWidth="17700" windowHeight="16605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ARI" sheetId="1" r:id="rId1"/>
     <sheet name="NMI" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -75,6 +88,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.0000_);[Red]\(0.0000\)"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -132,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -141,6 +157,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -448,14 +467,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="12.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.26953125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -466,301 +485,301 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="3">
-        <v>0.79500000000000004</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C5" s="4">
+        <v>0.58988387930835495</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="3">
-        <v>0.61070000000000002</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="4">
+        <v>0.22270059971328099</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="3">
-        <v>0.61070000000000002</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="4">
+        <v>0.22298713925637201</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="3">
-        <v>0.86929999999999996</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" s="4">
+        <v>0.69140214117952203</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="3">
-        <v>0.8881</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C9" s="4">
+        <v>0.70740373227489495</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="3">
-        <v>0.92220000000000002</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="4">
+        <v>0.79207920792079201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="3">
-        <v>0.83609999999999995</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C11" s="4">
+        <v>0.55685870754266498</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="3">
-        <v>0.9073</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="4">
+        <v>0.74988854213107503</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C13" s="3">
-        <v>0.9234</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C13" s="4">
+        <v>0.79336494457019202</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C14" s="3">
-        <v>0.66830000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C14" s="4">
+        <v>0.107953933914541</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="3">
-        <v>0.69240000000000002</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="4">
+        <v>0.175940816982953</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="3">
-        <v>0.6331</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C16" s="4">
+        <v>7.2669538660680003E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="3">
-        <v>0.90149999999999997</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="4">
+        <v>0.53901597328892903</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="3">
-        <v>0.99560000000000004</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C18" s="4">
+        <v>0.97712316059691495</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A19" s="3" t="s">
         <v>11</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="3">
-        <v>0.99560000000000004</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C19" s="4">
+        <v>0.97712316059691495</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C20" s="3">
-        <v>0.96250000000000002</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C20" s="4">
+        <v>0.842308885225028</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C21" s="3">
-        <v>0.92849999999999999</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C21" s="4">
+        <v>0.70393467918220398</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
         <v>12</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="3">
-        <v>0.93320000000000003</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C22" s="4">
+        <v>0.73001787338120505</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C23" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C23" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C24" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C24" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>13</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C25" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="3">
-        <v>0.55330000000000001</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C26" s="4">
+        <v>0.11052911751439499</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C27" s="3">
-        <v>0.58399999999999996</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C27" s="4">
+        <v>0.17011297709923701</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A28" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C28" s="3">
-        <v>0.5927</v>
+      <c r="C28" s="4">
+        <v>0.187282144835</v>
       </c>
     </row>
   </sheetData>
@@ -772,14 +791,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C28"/>
-  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.36328125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.375" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="1" customFormat="1" ht="14.25" x14ac:dyDescent="0.15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -790,7 +809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -801,7 +820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -812,7 +831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -823,7 +842,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
@@ -834,7 +853,7 @@
         <v>0.49130000000000001</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>7</v>
       </c>
@@ -845,7 +864,7 @@
         <v>0.2316</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
@@ -856,7 +875,7 @@
         <v>0.2515</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
@@ -867,7 +886,7 @@
         <v>0.88129999999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>8</v>
       </c>
@@ -878,7 +897,7 @@
         <v>0.7893</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
@@ -889,7 +908,7 @@
         <v>0.84570000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -900,7 +919,7 @@
         <v>0.61719999999999997</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
@@ -911,7 +930,7 @@
         <v>0.76429999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>9</v>
       </c>
@@ -922,7 +941,7 @@
         <v>0.80589999999999995</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>10</v>
       </c>
@@ -933,7 +952,7 @@
         <v>0.17330000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>10</v>
       </c>
@@ -944,7 +963,7 @@
         <v>0.26950000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>10</v>
       </c>
@@ -955,7 +974,7 @@
         <v>0.12770000000000001</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>11</v>
       </c>
@@ -966,7 +985,7 @@
         <v>0.70240000000000002</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
         <v>11</v>
       </c>
@@ -977,7 +996,7 @@
         <v>0.98119999999999996</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A19" s="3" t="s">
         <v>11</v>
       </c>
@@ -988,7 +1007,7 @@
         <v>0.98119999999999996</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
         <v>12</v>
       </c>
@@ -999,7 +1018,7 @@
         <v>0.88129999999999997</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
         <v>12</v>
       </c>
@@ -1010,7 +1029,7 @@
         <v>0.80259999999999998</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
         <v>12</v>
       </c>
@@ -1021,7 +1040,7 @@
         <v>0.8427</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>13</v>
       </c>
@@ -1032,7 +1051,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>13</v>
       </c>
@@ -1043,7 +1062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>13</v>
       </c>
@@ -1054,7 +1073,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
         <v>14</v>
       </c>
@@ -1065,7 +1084,7 @@
         <v>0.24079999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A27" s="3" t="s">
         <v>14</v>
       </c>
@@ -1076,7 +1095,7 @@
         <v>0.2137</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A28" s="3" t="s">
         <v>14</v>
       </c>

</xml_diff>